<commit_message>
fix(quick-11): repair Excel template formulas and white-card layout
Correct off-by-one row refs that caused #VALUE!, align defaults with
quick-11 (12M principal), and restyle the loan DTI workbook.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/downloads/quick11-loan-dti-template.xlsx
+++ b/assets/downloads/quick11-loan-dti-template.xlsx
@@ -40,7 +40,7 @@
     <t>NT$</t>
   </si>
   <si>
-    <t>例：120 萬</t>
+    <t>例：1200 萬</t>
   </si>
   <si>
     <t>年利率</t>
@@ -49,7 +49,7 @@
     <t>%</t>
   </si>
   <si>
-    <t>例：2.2</t>
+    <t>例：2.2（純數字，非文字）</t>
   </si>
   <si>
     <t>貸款年期</t>
@@ -58,7 +58,7 @@
     <t>年</t>
   </si>
   <si>
-    <t>例：30</t>
+    <t>例：30（純數字）</t>
   </si>
   <si>
     <t>月收入（預警）</t>
@@ -79,7 +79,7 @@
     <t>本息均攤 · 每月繳款</t>
   </si>
   <si>
-    <t>Excel PMT：固定月付</t>
+    <t>月利率 r＝年利率÷12÷100；n＝年期×12</t>
   </si>
   <si>
     <t>本金均攤 · 首期月付</t>
@@ -100,7 +100,7 @@
     <t>比率</t>
   </si>
   <si>
-    <t>建議 &lt;35% 較安全；&gt;50% 預警</t>
+    <t>建議 &lt;35% 較安全；≥50% 預警</t>
   </si>
   <si>
     <t>DTI 百分比</t>
@@ -109,10 +109,10 @@
     <t>破產計算機同款指標</t>
   </si>
   <si>
-    <t>破產預警文字</t>
-  </si>
-  <si>
-    <t>對照 quick-11 預警</t>
+    <t>財務健康狀態</t>
+  </si>
+  <si>
+    <t>DTI&gt;50% 自動顯示預警</t>
   </si>
   <si>
     <t>線上試算</t>
@@ -138,9 +138,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -150,30 +150,61 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF1E3A8A"/>
+      <color rgb="FF2D3748"/>
       <sz val="14"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF2D3748"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF0369A1"/>
+      <color rgb="FF4A5568"/>
+    </font>
+    <font>
+      <color rgb="FF2D3748"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF2563EB"/>
     </font>
     <font>
       <b/>
       <color rgb="FFB45309"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFDC2626"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF2563EB"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8F9FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0F4F8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -181,19 +212,74 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -534,15 +620,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -550,227 +636,245 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="3" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="2" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" ht="24" customHeight="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="3">
-        <v>1200000</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B5" s="8">
+        <v>12000000</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="9">
         <v>2.2</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="10">
         <v>30</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="8">
         <v>80000</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    <row r="9" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" ht="24" customHeight="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="13">
         <f>PMT(B6/12/100,B7*12,-B5)</f>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="12" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="14">
         <f>B5/(B7*12)+B5*B6/12/100</f>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="12" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="6">
-        <f>B11*B7*12-B5</f>
-      </c>
-      <c r="C14" t="s">
+      <c r="B14" s="14">
+        <f>B12*B7*12-B5</f>
+      </c>
+      <c r="C14" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="7">
-        <f>IF(B8=0,0,B11/B8)</f>
-      </c>
-      <c r="C15" t="s">
+      <c r="B15" s="15">
+        <f>IF(B8=0,0,B12/B8)</f>
+      </c>
+      <c r="C15" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="12" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B16">
-        <f>B14*100</f>
-      </c>
-      <c r="C16" t="s">
+      <c r="B16" s="16">
+        <f>B15*100</f>
+      </c>
+      <c r="C16" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="B17">
-        <f>IF(B15&gt;=50,"準備吃土：先降月付或拉高收入",IF(B15&gt;=35,"壓力偏高：月付偏緊","安全區：現金流尚可"))</f>
-      </c>
-      <c r="C17" t="s">
+      <c r="B17" s="18">
+        <f>IF(B16&gt;=50,"⚠ 破產預警：先降月付或拉高收入",IF(B16&gt;=35,"⚠ 壓力偏高：月付偏緊","✓ 安全區：現金流尚可"))</f>
+      </c>
+      <c r="C17" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="12" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="18" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="2" t="s">
         <v>39</v>
       </c>
     </row>
@@ -778,6 +882,10 @@
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B19" r:id="rId1"/>
+    <hyperlink ref="B20" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(quick-11): polish Excel template UI and reskin idle nudge card
Align loan DTI xlsx with dev excel-preview (white card, 微軟正黑體, A/C layout).
Reskin bottom idle nudge to premium dark layout; keep quick-1 triggers and CTA.
Remove accidental Excel lock file from downloads.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/downloads/quick11-loan-dti-template.xlsx
+++ b/assets/downloads/quick11-loan-dti-template.xlsx
@@ -11,17 +11,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
   <si>
     <t>破產計算機 · 貸款利息試算表（公式可改）</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>【輸入區】改 B 欄數字即可</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>項目</t>
   </si>
   <si>
@@ -49,7 +49,7 @@
     <t>%</t>
   </si>
   <si>
-    <t>例：2.2（純數字，非文字）</t>
+    <t>例：2.2 純數字</t>
   </si>
   <si>
     <t>貸款年期</t>
@@ -58,7 +58,7 @@
     <t>年</t>
   </si>
   <si>
-    <t>例：30（純數字）</t>
+    <t>例：30 純數字</t>
   </si>
   <si>
     <t>月收入（預警）</t>
@@ -79,13 +79,7 @@
     <t>本息均攤 · 每月繳款</t>
   </si>
   <si>
-    <t>月利率 r＝年利率÷12÷100；n＝年期×12</t>
-  </si>
-  <si>
-    <t>本金均攤 · 首期月付</t>
-  </si>
-  <si>
-    <t>首期＝本金攤還＋首期利息</t>
+    <t>PMT：月利率＝年利率÷12÷100</t>
   </si>
   <si>
     <t>本息均攤 · 總繳利息</t>
@@ -94,43 +88,13 @@
     <t>總付款－本金</t>
   </si>
   <si>
-    <t>DTI（月付／月收入）</t>
-  </si>
-  <si>
-    <t>比率</t>
-  </si>
-  <si>
-    <t>建議 &lt;35% 較安全；≥50% 預警</t>
-  </si>
-  <si>
-    <t>DTI 百分比</t>
-  </si>
-  <si>
-    <t>破產計算機同款指標</t>
+    <t>DTI 債務收入比</t>
+  </si>
+  <si>
+    <t>月付÷月收入；&lt;35% 安全；≥50% 預警</t>
   </si>
   <si>
     <t>財務健康狀態</t>
-  </si>
-  <si>
-    <t>DTI&gt;50% 自動顯示預警</t>
-  </si>
-  <si>
-    <t>線上試算</t>
-  </si>
-  <si>
-    <t>https://wealth-freedom-calculator.vercel.app/quick-11</t>
-  </si>
-  <si>
-    <t>手動輸入嫌麻煩可回站內試算</t>
-  </si>
-  <si>
-    <t>財富自由計算機</t>
-  </si>
-  <si>
-    <t>https://wealth-freedom-calculator.vercel.app/</t>
-  </si>
-  <si>
-    <t>長期 FIRE／股利課稅／54C 完整版</t>
   </si>
 </sst>
 </file>
@@ -138,9 +102,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0&quot;%&quot;"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -152,33 +116,53 @@
       <b/>
       <color rgb="FF2D3748"/>
       <sz val="14"/>
+      <name val="微軟正黑體"/>
     </font>
     <font>
       <b/>
       <color rgb="FF2D3748"/>
+      <sz val="11"/>
+      <name val="微軟正黑體"/>
     </font>
     <font>
       <b/>
       <color rgb="FF4A5568"/>
+      <sz val="11"/>
+      <name val="微軟正黑體"/>
     </font>
     <font>
       <color rgb="FF2D3748"/>
+      <sz val="11"/>
+      <name val="微軟正黑體"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF2563EB"/>
+      <color rgb="FF0284C7"/>
+      <sz val="11"/>
+      <name val="微軟正黑體"/>
+    </font>
+    <font>
+      <color rgb="FF4A5568"/>
+      <sz val="11"/>
+      <name val="微軟正黑體"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFB45309"/>
+      <color rgb="FF0369A1"/>
+      <sz val="11"/>
+      <name val="微軟正黑體"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFD97706"/>
+      <sz val="11"/>
+      <name val="微軟正黑體"/>
     </font>
     <font>
       <b/>
       <color rgb="FFDC2626"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF2563EB"/>
+      <sz val="11"/>
+      <name val="微軟正黑體"/>
     </font>
   </fonts>
   <fills count="5">
@@ -190,12 +174,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8F9FA"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFF8F9FA"/>
       </patternFill>
     </fill>
     <fill>
@@ -204,7 +188,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -227,64 +211,127 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFDC2626"/>
+        <sz val="11"/>
+        <name val="微軟正黑體"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFD97706"/>
+        <sz val="11"/>
+        <name val="微軟正黑體"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF7ED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF059669"/>
+        <sz val="11"/>
+        <name val="微軟正黑體"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -619,16 +666,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="38" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="56" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -636,256 +683,201 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
+    <row r="2" ht="12" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" ht="22" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
+    <row r="3" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="8">
         <v>12000000</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="11">
         <v>2.2</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="12">
         <v>30</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B8" s="8">
         <v>80000</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
+    <row r="9" ht="12" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" ht="22" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+    <row r="10" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+    <row r="12" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B12" s="13">
         <f>PMT(B6/12/100,B7*12,-B5)</f>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="10" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+    <row r="13" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="14">
-        <f>B5/(B7*12)+B5*B6/12/100</f>
-      </c>
-      <c r="C13" s="12" t="s">
+      <c r="B13" s="13">
+        <f>B12*B7*12-B5</f>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+    <row r="14" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>25</v>
       </c>
       <c r="B14" s="14">
-        <f>B12*B7*12-B5</f>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" s="12" t="s">
+        <f>IF(B8=0,0,B12/B8)</f>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+    <row r="15" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="15">
-        <f>IF(B8=0,0,B12/B8)</f>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" s="16">
-        <f>B15*100</f>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="18">
-        <f>IF(B16&gt;=50,"⚠ 破產預警：先降月付或拉高收入",IF(B16&gt;=35,"⚠ 壓力偏高：月付偏緊","✓ 安全區：現金流尚可"))</f>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-    </row>
-    <row r="19" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B20" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>39</v>
-      </c>
+      <c r="B15" s="16">
+        <f>IF(B14&gt;=0.5,"⚠ 破產預警：先降月付或拉高收入",IF(B14&gt;=0.35,"⚠ 壓力偏高：月付偏緊","✓ 安全區：現金流尚可"))</f>
+      </c>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+    </row>
+    <row r="16" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="7">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="A16:D16"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="B19" r:id="rId1"/>
-    <hyperlink ref="B20" r:id="rId2"/>
-  </hyperlinks>
+  <conditionalFormatting sqref="A15:D15">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$B$14&gt;=0.5</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>AND($B$14&gt;=0.35,$B$14&lt;0.5)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>$B$14&lt;0.35</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>